<commit_message>
Add annotated site maps, trailer staging model, and parking correction
Adds labelled aerial maps for the walking route, parking and trailer
staging, and the parade segment; models trailer and bus staging at the
candidate grass lot; corrects the parking lot to the open grass field
across from the high school, next to the fire station; and updates the
report and workbook to match.

Claude-Session: https://claude.ai/code/session_011hnYhedz3CwSoF8YU1nfPe
</commit_message>
<xml_diff>
--- a/deliverables/Caruthers_Showcase_Planning_Model.xlsx
+++ b/deliverables/Caruthers_Showcase_Planning_Model.xlsx
@@ -702,7 +702,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Share of football-field parking used by the fair on Saturday (assumed)</t>
+          <t>Share of the open grass lot used by the fair on Saturday (assumed)</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Football-field parking spaces (unverified, to measure)</t>
+          <t>Open grass lot across from the high school, used for fair parking, next to the fire station (unverified, to measure)</t>
         </is>
       </c>
     </row>

</xml_diff>